<commit_message>
Add automatic lead finder and improved Excel template
- find_leads.py: searches Google Maps Places API for businesses with
  no website in any city/industry, exports ready-to-use Excel
- leads_template.xlsx: tip row added for each column, owner_name
  marked as optional (defaults to 'Hi there' in email)

https://claude.ai/code/session_01RtM7kMpXXJpnPzwJkqWXkZ
</commit_message>
<xml_diff>
--- a/outreach/leads_template.xlsx
+++ b/outreach/leads_template.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,8 +29,13 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <i val="1"/>
+      <color rgb="000D1B2A"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -41,6 +46,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="000D1B2A"/>
         <bgColor rgb="000D1B2A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5A623"/>
+        <bgColor rgb="00F5A623"/>
       </patternFill>
     </fill>
   </fills>
@@ -56,10 +67,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -426,12 +440,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="26" customWidth="1" min="6" max="6"/>
@@ -439,7 +453,7 @@
     <col width="34" customWidth="1" min="8" max="8"/>
     <col width="40" customWidth="1" min="9" max="9"/>
     <col width="40" customWidth="1" min="10" max="10"/>
-    <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="50" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -499,56 +513,60 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Rodriguez Plumbing</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Carlos Rodriguez</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>plumber</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Los Angeles</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>CA</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>carlos@example.com</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>(323) 555-0101</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>142 Main St, Los Angeles, CA 90012</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>https://maps.google.com/?cid=123</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Emergency callouts 24/7, family run since 2005</t>
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>e.g. Rodriguez Plumbing</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Leave blank if unknown — defaults to Hi there</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>plumber / cleaner / landscaper / roofer / electrician / painter / hvac / handyman</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>e.g. Manchester</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>e.g. CA or leave blank for UK</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Required for sending</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>e.g. 07700 900123</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Full street address for footer of mock site</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Paste direct image URL of their logo (optional)</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Google Maps link (optional)</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Any extra context: family run, 20 yrs exp, emergency callouts...</t>
         </is>
       </c>
     </row>
@@ -558,11 +576,7 @@
           <t>Green Lawn Care</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Mike Johnson</t>
-        </is>
-      </c>
+      <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
           <t>landscaper</t>
@@ -570,14 +584,10 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Austin</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>TX</t>
-        </is>
-      </c>
+          <t>Manchester</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>mike@example.com</t>
@@ -585,64 +595,23 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>(512) 555-0187</t>
+          <t>07700 900187</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>89 Oak Ave, Austin, TX 78701</t>
+          <t>89 Oak Ave, Manchester M1 2AB</t>
         </is>
       </c>
       <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>https://maps.google.com/?cid=456</t>
+        </is>
+      </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Residential and commercial, free quotes</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Sparkle Clean Co</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Sarah Williams</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>cleaning</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Manchester</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>sarah@example.com</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>07700 900123</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>15 Brook St, Manchester, M1 2AB</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>End of tenancy specialist</t>
+          <t>Residential, free quotes, serves all of Manchester</t>
         </is>
       </c>
     </row>

</xml_diff>